<commit_message>
verifier assignment flow and document upload with template data
</commit_message>
<xml_diff>
--- a/public/assets/excel_formats/sampleTemplate.xlsx
+++ b/public/assets/excel_formats/sampleTemplate.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="16">
   <si>
     <t>Sr</t>
   </si>
@@ -57,6 +57,12 @@
   </si>
   <si>
     <t>Yes / No</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>Column4</t>
   </si>
 </sst>
 </file>
@@ -487,8 +493,18 @@
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="C5"/>
-      <c r="E5"/>
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="C6"/>
@@ -1272,8 +1288,8 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="C2:C200">
-      <formula1>"Free Text,Dropdown,Yes / No"</formula1>
+    <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" promptTitle="Type" prompt="File: each cell of this column holds one file name (e.g. abc.pdf) or one link." sqref="C2:C200">
+      <formula1>"Free Text,Dropdown,Yes / No,File"</formula1>
     </dataValidation>
     <dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" sqref="E2:E200">
       <formula1>"Yes,No"</formula1>

</xml_diff>